<commit_message>
Ingest batch 1 (7/10): real подряд cases + verified NOSTROY statuses
ЮГСЕРВИС & ДДК confirmed 'Приостановлено'; Ростгорсвет & ЮГСЕРВИС ОДО
не установлен. 34 подряд-cases 2025+ across 7 companies.
</commit_message>
<xml_diff>
--- a/audit/audit_report_corrected.xlsx
+++ b/audit/audit_report_corrected.xlsx
@@ -491,7 +491,7 @@
     <row r="1" ht="95" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 2/67; дела проверены: 0/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 2, ОДО не установлен: 1. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 11, Средний: 0, Низкий: 0, Ожидает: 56.</t>
+          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 7/67; дела проверены: 7/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 2, ОДО не установлен: 2. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 14, Средний: 0, Низкий: 0, Ожидает: 53.</t>
         </is>
       </c>
     </row>
@@ -586,23 +586,25 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Третий уровень</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>11</v>
+      </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-17506/2026 — 53 331 ₽ — ответчик; А53-16758/2026 — 0 ₽ — истец; А53-15623/2026 — 590 000 ₽ — третье лицо; А53-15343/2026 — 38 015 541 ₽ — истец; А53-11758/2026 — 54 713 831 ₽ — истец; А53-46207/2025 — 10 947 592 ₽ — истец; А53-31277/2025 — 413 951 ₽ — истец; А53-31468/2025 — 3 398 681 ₽ — истец; А53-17979/2025 — 1 477 015 ₽ — истец; А53-17976/2025 — 229 999 ₽ — истец; А53-12185/2025 — 75 027 ₽ — истец</t>
         </is>
       </c>
       <c r="K3" s="4" t="n">
@@ -615,7 +617,7 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 60 509 176 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (11); крупные штрафы/неустойки 60 509 176 ₽</t>
         </is>
       </c>
     </row>
@@ -643,36 +645,38 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Третий уровень</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-16432/2026 — 2 035 549 ₽ — истец; А53-16444/2026 — 2 995 500 ₽ — истец; А53-16485/2026 — 278 832 ₽ — истец; А53-48319/2025 — 2 948 572 ₽ — ответчик; А53-31499/2025 — 489 000 ₽ — ответчик; А53-1777/2025 — 122 230 ₽ — третье лицо</t>
         </is>
       </c>
       <c r="K4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>арбитражные дела по подряду 2025+ (6)</t>
         </is>
       </c>
     </row>
@@ -700,36 +704,38 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>не установлен</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-46162/2025 — 74 200 ₽ — истец; А53-9899/2025 — 4 261 841 ₽ — ответчик</t>
         </is>
       </c>
       <c r="K5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (2)</t>
         </is>
       </c>
     </row>
@@ -757,23 +763,25 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Четвертый уровень</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-18293/2026 — 11 480 558 ₽ — ответчик; А19-3283/2026 — 0 ₽ — ответчик; А19-2654/2026 — 11 480 557 ₽ — ответчик; А19-353/2026 — 703 237 ₽ — ответчик; А19-21740/2025 — 22 556 385 ₽ — истец; А19-11465/2025 — 0 ₽ — третье лицо; А19-3476/2025 — 115 647 ₽ — истец</t>
         </is>
       </c>
       <c r="K6" s="4" t="n">
@@ -786,7 +794,7 @@
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 1 339 858 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (7); крупные штрафы/неустойки 1 339 858 ₽</t>
         </is>
       </c>
     </row>
@@ -814,36 +822,38 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Четвертый уровень</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-46084/2025 — 3 581 250 ₽ — истец; А53-34365/2025 — 9 891 254 ₽ — истец; А53-34092/2025 — 81 593 177 ₽ — ответчик; А53-26845/2025 — 1 167 795 ₽ — истец; А53-21492/2025 — 968 150 ₽ — истец</t>
         </is>
       </c>
       <c r="K7" s="4" t="n">
         <v>28566.76</v>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены; небольшие штрафы/неустойки 28 567 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (5)</t>
         </is>
       </c>
     </row>
@@ -928,7 +938,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>приостановлен</t>
+          <t>Приостановлено</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -938,13 +948,15 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-44550/2025 — 188 836 ₽ — ответчик; А53-30087/2025 — 986 882 ₽ — ответчик; А83-11057/2025 — 92 378 562 ₽ — третье лицо</t>
         </is>
       </c>
       <c r="K9" s="4" t="n">
@@ -957,7 +969,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; уровень ответственности (ОДО) не установлен; крупные штрафы/неустойки 2 485 954 ₽</t>
+          <t>статус НОСТРОЙ приостановлен; уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (3); крупные штрафы/неустойки 2 485 954 ₽</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1339,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>приостановлен</t>
+          <t>Приостановлено</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1337,13 +1349,15 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-13038/2026 — 2 126 623 ₽ — ответчик</t>
         </is>
       </c>
       <c r="K16" s="4" t="n">
@@ -1356,7 +1370,7 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6191,16 +6205,2161 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>⏳ Дела по подряду ещё не собраны по полному источнику (kad.arbitr.ru). Rusprofile показывает категории дел только по платной подписке.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>А53-17506/2026</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>07.05.2026</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Рба-МБ"</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>53330.67</v>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/30c3feee-3c5f-458a-b892-db0fbabf92e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>А53-16758/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>04.05.2026</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>ГУП РО "Урсв"</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/d11b7613-cce1-4de8-bc15-497a5995f04c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>А53-15623/2026</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>23.04.2026</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Дсигр</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Генпроект"</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт" (третье лицо), Диара, Росстройконтроль</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>третье лицо</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>590000</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/8954e61f-2f0e-475a-96c7-f4df9a08ff22</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>А53-15343/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>22.04.2026</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Министерство Строительства РО</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>38015541.37</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/fc09e91a-fec5-481f-ba0a-e8d75d204808</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>А53-11758/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>30.03.2026</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>МКУ "Отдел Заказчика" Боковского района</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>54713831.07</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/08b38eb7-d44e-443d-b117-899e902d860b</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>А53-46207/2025</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>04.12.2025</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройгазсервис"</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>10947592.32</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/e7054f47-51e3-46c7-a748-acbd5e9f4e84</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>А53-31277/2025</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>28.08.2025</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>ИП Крот М.М.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>413950.68</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Частично выиграно</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/2fff797b-51b8-4d2a-802c-07f601237217</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>А53-31468/2025</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>28.08.2025</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Министерство ЖКХ области</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>иное лицо ГБУ РО "Ростовоблстройзаказчик"</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>3398681.18</v>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/da4da002-645c-4d09-9009-c11c2b66085c</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>А53-17979/2025</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>26.05.2025</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>ИП Васильцова Н.В.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>1477014.66</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Не выиграно</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/1b94b99c-1b87-4f52-af8f-dd4edf56452c</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>А53-17976/2025</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>26.05.2025</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>ИП Радченко А.А.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>229999.45</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Не выиграно</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/e33c4534-40c3-4550-9baa-c07131ff7038</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ЛИМЕРТ</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>6154148600</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>А53-12185/2025</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>09.04.2025</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Лимерт"</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>ООО РТЗ "Спецстрой"</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>75026.59</v>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Выиграно</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/28800f26-846e-49de-a02b-d9f1460e25f8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>6163212700</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>А53-16432/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>29.04.2026</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Цифровое Превосходство"</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Су-5"</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>2035549.14</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/7050a254-57fd-4eb0-abef-c9d0a44c5bd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>6163212700</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>А53-16444/2026</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>29.04.2026</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Цифровое Превосходство"</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>АО "Апск "ГСА"</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>2995500</v>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/ead99d04-0c07-43d6-9d73-c42df831373f</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>6163212700</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>А53-16485/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>29.04.2026</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Цифровое Превосходство"</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Нор-Девелопмент"</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>278832.19</v>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/70a699b6-70ce-4380-ae65-f6178d036756</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>6163212700</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>А53-48319/2025</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>16.12.2025</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Цифровоепревосходство", ООО "Мономер-Т"</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Цифровое Превосходство"</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>2948572</v>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Не проиграно</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/3baabdf8-d91b-4fa1-8510-7a8452e1f586</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>6163212700</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>А53-31499/2025</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>29.08.2025</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>ИП Денисов Д.В.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Цифровое Превосходство"</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>489000</v>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Проиграно</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/409242c8-b063-4bf7-82ee-cd313dbcf242</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>6163212700</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>А53-1777/2025</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>24.01.2025</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>МБУ "Центр ИТС"</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Акгёзова Аида Бийисламовна</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Цифровое Превосходство" (третье лицо), Муниципальное Казначейство; иное лицо Хасанов Р.И.</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>третье лицо</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>122229.75</v>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>В роли третьего/иного лица</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/79a4f003-5b4d-4674-8b2d-44cca7e7a30f</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Ростгорсвет</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>6164246452</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>А53-46162/2025</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>04.12.2025</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>МКП "Ростгорсвет"</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>ИП Майоров М.В.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>74200.42999999999</v>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Не выиграно</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/7ab9cf32-c281-4b0c-89d3-971592da5280</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Ростгорсвет</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>6164246452</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>А53-9899/2025</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>25.03.2025</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>ИП Ковальчук А.В.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>МКП "Ростгорсвет"</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>4261840.97</v>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Частично проиграно</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/2fd1d200-767f-49cb-a077-641ab2a71f93</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>СТРОЙДОРХОЛДИНГ</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>3810050189</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>А53-18293/2026</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>14.05.2026</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>ООО РСП "Топка"</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройдорхолдинг"</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>11480557.63</v>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/5515b5e6-d533-4e44-8b6b-ff34305adf25</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>СТРОЙДОРХОЛДИНГ</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>3810050189</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>А19-3283/2026</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>11.02.2026</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>КГХ Администрации Города Усолье-Сибирское</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройдорхолдинг"</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Не проиграно</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/fdfea6c1-42e3-4cac-bc9a-79ba989a16f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>СТРОЙДОРХОЛДИНГ</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>3810050189</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>А19-2654/2026</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>04.02.2026</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>ООО РСП "Топка"</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройдорхолдинг"</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>11480557</v>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Прекращено</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/dd04508a-5cd5-4d41-b5c8-7e183e33a149</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>СТРОЙДОРХОЛДИНГ</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>3810050189</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>А19-353/2026</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>13.01.2026</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>КГХ Усолье-Сибирское</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройдорхолдинг"</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>703237</v>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Проиграно</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/3cf7d9eb-a9d6-4a7f-afe0-2429fc73e563</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>СТРОЙДОРХОЛДИНГ</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>3810050189</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>А19-21740/2025</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>16.09.2025</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройдорхолдинг"</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>АО "ДСК 156"</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>22556385</v>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Выиграно</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/6d66d0bd-99d0-4111-a68d-db241a8d24a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>СТРОЙДОРХОЛДИНГ</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>3810050189</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>А19-11465/2025</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>23.05.2025</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>отсутствует</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Комитет по ЖКХ</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройдорхолдинг" (третье лицо)</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>третье лицо</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/b66d7d66-4990-4bbe-bc6a-db88b4ea36e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>СТРОЙДОРХОЛДИНГ</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>3810050189</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>А19-3476/2025</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>17.02.2025</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройдорхолдинг"</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ПКФ "Пионер"</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>115647</v>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Выиграно</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/8ebed499-598d-49e0-9c44-f73a35642e77</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>ЮСК</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>6167073060</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>А53-46084/2025</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>03.12.2025</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ЮСК"</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Русалексгрупп"</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>3581250</v>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/b1b8c0e5-ed0f-4ed2-ba60-f608da312c09</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>ЮСК</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>6167073060</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>А53-34365/2025</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>18.09.2025</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ЮСК"</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>ООО "МФС Групп"</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>9891254.279999999</v>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Не выиграно</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/167ea3b1-7b52-4c91-94dc-68db6bda757b</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>ЮСК</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>6167073060</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>А53-34092/2025</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>17.09.2025</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>МКУ "УКС"</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ЮСК"</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>81593176.87</v>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Не проиграно</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/f9f5665f-5a2e-408f-bffa-bc8adecb44ec</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>ЮСК</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>6167073060</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>А53-26845/2025</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>28.07.2025</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ЮСК"</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>ИП Янковская К.О.</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>1167795.4</v>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Выиграно</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/84d1e8bb-d21a-415b-b5dc-f1ee54963268</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>ЮСК</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>6167073060</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>А53-21492/2025</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>23.06.2025</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ЮСК"</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>ИП Янковская К.О.</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>968150</v>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Прекращено</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/41f4a8ef-a888-4315-8e6f-1cda1308724d</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>ОООЮГСЕРВИС</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>6167127284</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>А53-44550/2025</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>25.11.2025</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Дока-Строй"</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Югсервис"</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>188835.64</v>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Проиграно</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/2f9675d6-5d72-4211-bdde-90645c9a23f8</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>ОООЮГСЕРВИС</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>6167127284</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>А53-30087/2025</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>19.08.2025</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Дока-Строй"</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Югсервис"</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>986882.5</v>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Проиграно</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/9d82aa5e-4a38-4925-8048-0ae5d3f4fb21</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>ОООЮГСЕРВИС</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>6167127284</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>А83-11057/2025</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>04.06.2025</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>ООО "СТИ"</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>ГКУ "Инвестстрой Республики Крым"</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Югсервис", Банк ВТБ, КФУ; иное лицо Губайдулин А.М.</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>третье лицо</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>92378561.65000001</v>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>В роли третьего/иного лица</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/9b484cdb-1097-4cb0-ac24-e24ff3df04a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>КОМПАНИЯ ДДК</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>6168081843</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>А53-13038/2026</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Юнас+"</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Компания ДДК"</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>2126622.87</v>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/0e4a3044-7540-437e-b6b0-2bf087d604c3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:M2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6284,21 +8443,23 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr"/>
+          <t>Третий уровень</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>11</v>
+      </c>
       <c r="G2" s="4" t="n">
         <v>60509176.12</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 60 509 176 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (11); крупные штрафы/неустойки 60 509 176 ₽</t>
         </is>
       </c>
     </row>
@@ -6320,21 +8481,23 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr"/>
+          <t>Четвертый уровень</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="G3" s="4" t="n">
         <v>1339858.11</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 1 339 858 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (7); крупные штрафы/неустойки 1 339 858 ₽</t>
         </is>
       </c>
     </row>
@@ -6346,31 +8509,33 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ПСС</t>
+          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>6163226020</t>
+          <t>6163212700</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
+          <t>Третий уровень</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="G4" s="4" t="n">
-        <v>20712302.61</v>
+        <v>0</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 20 712 303 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (6)</t>
         </is>
       </c>
     </row>
@@ -6382,31 +8547,33 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>ОООЮГСЕРВИС</t>
+          <t>ЮСК</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>6167127284</t>
+          <t>6167073060</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>приостановлен</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
+          <t>Четвертый уровень</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="G5" s="4" t="n">
-        <v>2485954.43</v>
+        <v>28566.76</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; уровень ответственности (ОДО) не установлен; крупные штрафы/неустойки 2 485 954 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (5)</t>
         </is>
       </c>
     </row>
@@ -6418,31 +8585,33 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>СУ-310</t>
+          <t>ОООЮГСЕРВИС</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>6167126523</t>
+          <t>6167127284</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Приостановлено</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr"/>
+          <t>не установлен</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G6" s="4" t="n">
-        <v>10372474.95</v>
+        <v>2485954.43</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 10 372 475 ₽</t>
+          <t>статус НОСТРОЙ приостановлен; уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (3); крупные штрафы/неустойки 2 485 954 ₽</t>
         </is>
       </c>
     </row>
@@ -6454,31 +8623,33 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>КОМПАНИЯ ДДК</t>
+          <t>Ростгорсвет</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>6168081843</t>
+          <t>6164246452</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>приостановлен</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
+          <t>не установлен</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен</t>
+          <t>уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (2)</t>
         </is>
       </c>
     </row>
@@ -6490,31 +8661,33 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ростовстрой</t>
+          <t>КОМПАНИЯ ДДК</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>6166125510</t>
+          <t>6168081843</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Приостановлено</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr"/>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="G8" s="4" t="n">
-        <v>1231653.69</v>
+        <v>0</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 1 231 654 ₽</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>
@@ -6526,12 +8699,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>ЭНТЭЛ</t>
+          <t>ПСС</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>6163214264</t>
+          <t>6163226020</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -6546,11 +8719,11 @@
       </c>
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="4" t="n">
-        <v>4691800.99</v>
+        <v>20712302.61</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 4 691 801 ₽</t>
+          <t>крупные штрафы/неустойки 20 712 303 ₽</t>
         </is>
       </c>
     </row>
@@ -6562,12 +8735,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>СТРОЙГАРАНТ</t>
+          <t>СУ-310</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>9204000968</t>
+          <t>6167126523</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -6582,11 +8755,11 @@
       </c>
       <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="4" t="n">
-        <v>3657989.45</v>
+        <v>10372474.95</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 3 657 989 ₽</t>
+          <t>крупные штрафы/неустойки 10 372 475 ₽</t>
         </is>
       </c>
     </row>
@@ -6598,12 +8771,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Ресурс-Дон</t>
+          <t>Ростовстрой</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>6163138292</t>
+          <t>6166125510</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -6618,11 +8791,11 @@
       </c>
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="4" t="n">
-        <v>18336806.38</v>
+        <v>1231653.69</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 18 336 806 ₽</t>
+          <t>крупные штрафы/неустойки 1 231 654 ₽</t>
         </is>
       </c>
     </row>
@@ -6634,12 +8807,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>АМЕТИСТ</t>
+          <t>ЭНТЭЛ</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>6165157340</t>
+          <t>6163214264</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -6654,28 +8827,28 @@
       </c>
       <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="4" t="n">
-        <v>1032995.69</v>
+        <v>4691800.99</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 1 032 996 ₽</t>
+          <t>крупные штрафы/неустойки 4 691 801 ₽</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ЦИФРОВОЕ ПРЕВОСХОДСТВО</t>
+          <t>СТРОЙГАРАНТ</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>6163212700</t>
+          <t>9204000968</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -6690,28 +8863,28 @@
       </c>
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="4" t="n">
-        <v>0</v>
+        <v>3657989.45</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>крупные штрафы/неустойки 3 657 989 ₽</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Ростгорсвет</t>
+          <t>Ресурс-Дон</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>6164246452</t>
+          <t>6163138292</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -6726,28 +8899,28 @@
       </c>
       <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>18336806.38</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>крупные штрафы/неустойки 18 336 806 ₽</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>ЮСК</t>
+          <t>АМЕТИСТ</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>6167073060</t>
+          <t>6165157340</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -6762,11 +8935,11 @@
       </c>
       <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="4" t="n">
-        <v>28566.76</v>
+        <v>1032995.69</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены; небольшие штрафы/неустойки 28 567 ₽</t>
+          <t>крупные штрафы/неустойки 1 032 996 ₽</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete batch 1 (10/10 companies, 46 подряд cases); optimize extension command
- Ingest ПСС, Полимерспецстрой, ПКТ
- Add speed+accuracy guidance; instruct extension to take kad_url from
  Rusprofile's «На сайте КАД» href instead of loading kad.arbitr.ru pages
</commit_message>
<xml_diff>
--- a/audit/audit_report_corrected.xlsx
+++ b/audit/audit_report_corrected.xlsx
@@ -491,7 +491,7 @@
     <row r="1" ht="95" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 7/67; дела проверены: 7/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 2, ОДО не установлен: 2. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 14, Средний: 0, Низкий: 0, Ожидает: 53.</t>
+          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 10/67; дела проверены: 10/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 2, ОДО не установлен: 2. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 16, Средний: 0, Низкий: 0, Ожидает: 51.</t>
         </is>
       </c>
     </row>
@@ -881,23 +881,25 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А05-2918/2026 — 645 216 ₽ — ответчик; А53-3691/2026 — 19 379 993 ₽ — истец; А53-50381/2025 — 42 130 977 ₽ — ответчик; А53-24171/2025 — 13 293 113 ₽ — ответчик</t>
         </is>
       </c>
       <c r="K8" s="4" t="n">
@@ -910,7 +912,7 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 20 712 303 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (4); крупные штрафы/неустойки 20 712 303 ₽</t>
         </is>
       </c>
     </row>
@@ -997,36 +999,38 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Третий уровень</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А53-15589/2026 — 19 692 413 ₽ — ответчик; А53-46577/2025 — 0 ₽ — истец; А53-22788/2025 — 0 ₽ — ответчик; А53-12447/2025 — 5 400 633 ₽ — ответчик</t>
         </is>
       </c>
       <c r="K10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>арбитражные дела по подряду 2025+ (4)</t>
         </is>
       </c>
     </row>
@@ -1054,36 +1058,38 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr"/>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>А40-47154/2026 — 1 830 150 ₽ — ответчик; А53-15234/2025 — 4 820 741 ₽ — истец; А53-8542/2025 — 309 220 ₽ — истец</t>
         </is>
       </c>
       <c r="K11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>арбитражные дела по подряду 2025+ (3)</t>
         </is>
       </c>
     </row>
@@ -6119,7 +6125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8114,37 +8120,37 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>ОООЮГСЕРВИС</t>
+          <t>ПСС</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>6167127284</t>
+          <t>6163226020</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>А53-44550/2025</t>
+          <t>А05-2918/2026</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>18.03.2026</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+          <t>Подряд - неисполнение или ненадлежащее исполнение обязательств</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>ООО "Дока-Строй"</t>
+          <t>ИП Федькович А.В.</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>ООО "Югсервис"</t>
+          <t>ООО "ПСС"</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -8154,11 +8160,11 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>188835.64</v>
+        <v>645216.12</v>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Проиграно</t>
+          <t>Частично проиграно</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
@@ -8168,29 +8174,29 @@
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/2f9675d6-5d72-4211-bdde-90645c9a23f8</t>
+          <t>https://kad.arbitr.ru/Card/879a3093-8e76-49ab-8fc1-41d556003753</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>ОООЮГСЕРВИС</t>
+          <t>ПСС</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>6167127284</t>
+          <t>6163226020</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>А53-30087/2025</t>
+          <t>А53-3691/2026</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -8200,26 +8206,26 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>ООО "Дока-Строй"</t>
+          <t>ООО "ПСС"</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>ООО "Югсервис"</t>
+          <t>ООО "Союздонстрой"</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>ответчик</t>
+          <t>истец</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>986882.5</v>
+        <v>19379992.99</v>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Проиграно</t>
+          <t>Не выиграно</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
@@ -8229,131 +8235,810 @@
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/9d82aa5e-4a38-4925-8048-0ae5d3f4fb21</t>
+          <t>https://kad.arbitr.ru/Card/8cab0f29-4a76-4cf4-966e-c57e412e2028</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>ОООЮГСЕРВИС</t>
+          <t>ПСС</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>6167127284</t>
+          <t>6163226020</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>А83-11057/2025</t>
+          <t>А53-50381/2025</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>04.06.2025</t>
+          <t>26.12.2025</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>ООО "СТИ"</t>
+          <t>ООО "Артель"</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>ГКУ "Инвестстрой Республики Крым"</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>ООО "Югсервис", Банк ВТБ, КФУ; иное лицо Губайдулин А.М.</t>
-        </is>
-      </c>
+          <t>ООО "ПСС"</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>третье лицо</t>
+          <t>ответчик</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>92378561.65000001</v>
+        <v>42130977.24</v>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>В роли третьего/иного лица</t>
+          <t>Рассматривается</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>Завершено</t>
+          <t>Рассматривается</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/9b484cdb-1097-4cb0-ac24-e24ff3df04a9</t>
+          <t>https://kad.arbitr.ru/Card/7add7d5a-3c6a-4b9b-9364-27d943ceb8b2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
+          <t>ПСС</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>6163226020</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>А53-24171/2025</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>08.07.2025</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>МКУ "УКС"</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ПСС"</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Сим Пласт", Копченко А.М. (третьи лица); иное лицо ООО "Артель"</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>13293112.74</v>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/0bc93eeb-ab4e-428f-a1ee-e032380ee6a0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>ОООЮГСЕРВИС</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>6167127284</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>А53-44550/2025</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>25.11.2025</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Дока-Строй"</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Югсервис"</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>188835.64</v>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Проиграно</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/2f9675d6-5d72-4211-bdde-90645c9a23f8</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>ОООЮГСЕРВИС</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>6167127284</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>А53-30087/2025</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>19.08.2025</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Дока-Строй"</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Югсервис"</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>986882.5</v>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Проиграно</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/9d82aa5e-4a38-4925-8048-0ae5d3f4fb21</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>ОООЮГСЕРВИС</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>6167127284</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>А83-11057/2025</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>04.06.2025</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>ООО "СТИ"</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>ГКУ "Инвестстрой Республики Крым"</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Югсервис", Банк ВТБ, КФУ; иное лицо Губайдулин А.М.</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>третье лицо</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>92378561.65000001</v>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>В роли третьего/иного лица</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/9b484cdb-1097-4cb0-ac24-e24ff3df04a9</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>ОООПолимерспецстрой</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>6155050037</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>А53-15589/2026</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>23.04.2026</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Дельта-Л"</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Полимерспецстрой"</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>19692413.4</v>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/217123e5-7393-4e49-b43c-ab2c75b347bf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>ОООПолимерспецстрой</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>6155050037</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>А53-46577/2025</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>05.12.2025</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Полимерспецстрой"</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Управление ЖКХ Г. Азова</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/620a7b0b-42dd-44ac-928a-64cade291e06</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>ОООПолимерспецстрой</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>6155050037</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>А53-22788/2025</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>01.07.2025</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>МКУ "Департамент ГХ"</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Полимерспецстрой"</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>ООО Экспертное Бюро "Верум", ООО "Армила" (третьи лица); иное лицо ГУП РО "Урсв"</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/ffbf94a6-e419-4ec2-8928-27639ae26841</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>ОООПолимерспецстрой</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>6155050037</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>А53-12447/2025</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>10.04.2025</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Высокая Марка"</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Полимерспецстрой"</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>5400633.19</v>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/83e45950-1538-40dc-b570-1a0931c94a17</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>ОООПКТ</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>6168032645</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>А40-47154/2026</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>ООО "В2В"</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ПКТ"</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>1830150</v>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>Рассматривается</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/a38e254c-cb38-4b47-aeda-dcf1712c13d2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>ОООПКТ</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>6168032645</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>А53-15234/2025</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>30.04.2025</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ПКТ"</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Ростстройком"</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>4820741.07</v>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Не выиграно</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/c134956b-f62a-40ec-8f72-e8a215e9c076</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>ОООПКТ</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>6168032645</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>А53-8542/2025</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>17.03.2025</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>ООО "ПКТ"</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Ростстройком"</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>истец</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>309219.73</v>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Частично выиграно</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/de300706-4c42-4c61-a3fd-57c8a352886f</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
           <t>КОМПАНИЯ ДДК</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>6168081843</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>А53-13038/2026</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>07.04.2026</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F47" s="3" t="inlineStr">
         <is>
           <t>ООО "Юнас+"</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>ООО "Компания ДДК"</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr">
         <is>
           <t>ответчик</t>
         </is>
       </c>
-      <c r="J36" s="4" t="n">
+      <c r="J47" s="4" t="n">
         <v>2126622.87</v>
       </c>
-      <c r="K36" s="3" t="inlineStr">
+      <c r="K47" s="3" t="inlineStr">
         <is>
           <t>Рассматривается</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr">
+      <c r="L47" s="3" t="inlineStr">
         <is>
           <t>Рассматривается</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr">
+      <c r="M47" s="3" t="inlineStr">
         <is>
           <t>https://kad.arbitr.ru/Card/0e4a3044-7540-437e-b6b0-2bf087d604c3</t>
         </is>
@@ -8585,33 +9270,33 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ОООЮГСЕРВИС</t>
+          <t>ПСС</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>6167127284</t>
+          <t>6163226020</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Приостановлено</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2485954.43</v>
+        <v>20712302.61</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (3); крупные штрафы/неустойки 2 485 954 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (4); крупные штрафы/неустойки 20 712 303 ₽</t>
         </is>
       </c>
     </row>
@@ -8623,12 +9308,12 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Ростгорсвет</t>
+          <t>ОООПолимерспецстрой</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>6164246452</t>
+          <t>6155050037</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -8638,18 +9323,18 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Третий уровень</t>
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (2)</t>
+          <t>арбитражные дела по подряду 2025+ (4)</t>
         </is>
       </c>
     </row>
@@ -8661,12 +9346,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>КОМПАНИЯ ДДК</t>
+          <t>ОООЮГСЕРВИС</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>6168081843</t>
+          <t>6167127284</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -8676,18 +9361,18 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
+          <t>не установлен</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0</v>
+        <v>2485954.43</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
+          <t>статус НОСТРОЙ приостановлен; уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (3); крупные штрафы/неустойки 2 485 954 ₽</t>
         </is>
       </c>
     </row>
@@ -8699,31 +9384,33 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>ПСС</t>
+          <t>ОООПКТ</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>6163226020</t>
+          <t>6168032645</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr"/>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="G9" s="4" t="n">
-        <v>20712302.61</v>
+        <v>0</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 20 712 303 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (3)</t>
         </is>
       </c>
     </row>
@@ -8735,31 +9422,33 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>СУ-310</t>
+          <t>Ростгорсвет</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>6167126523</t>
+          <t>6164246452</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Действителен</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr"/>
+          <t>не установлен</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="G10" s="4" t="n">
-        <v>10372474.95</v>
+        <v>0</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 10 372 475 ₽</t>
+          <t>уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (2)</t>
         </is>
       </c>
     </row>
@@ -8771,31 +9460,33 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Ростовстрой</t>
+          <t>КОМПАНИЯ ДДК</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>6166125510</t>
+          <t>6168081843</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Приостановлено</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="G11" s="4" t="n">
-        <v>1231653.69</v>
+        <v>0</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 1 231 654 ₽</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>
@@ -8807,12 +9498,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ЭНТЭЛ</t>
+          <t>СУ-310</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>6163214264</t>
+          <t>6167126523</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -8827,11 +9518,11 @@
       </c>
       <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="4" t="n">
-        <v>4691800.99</v>
+        <v>10372474.95</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 4 691 801 ₽</t>
+          <t>крупные штрафы/неустойки 10 372 475 ₽</t>
         </is>
       </c>
     </row>
@@ -8843,12 +9534,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>СТРОЙГАРАНТ</t>
+          <t>Ростовстрой</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>9204000968</t>
+          <t>6166125510</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -8863,11 +9554,11 @@
       </c>
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="4" t="n">
-        <v>3657989.45</v>
+        <v>1231653.69</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 3 657 989 ₽</t>
+          <t>крупные штрафы/неустойки 1 231 654 ₽</t>
         </is>
       </c>
     </row>
@@ -8879,12 +9570,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Ресурс-Дон</t>
+          <t>ЭНТЭЛ</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>6163138292</t>
+          <t>6163214264</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -8899,11 +9590,11 @@
       </c>
       <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="4" t="n">
-        <v>18336806.38</v>
+        <v>4691800.99</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 18 336 806 ₽</t>
+          <t>крупные штрафы/неустойки 4 691 801 ₽</t>
         </is>
       </c>
     </row>
@@ -8915,12 +9606,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>АМЕТИСТ</t>
+          <t>СТРОЙГАРАНТ</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>6165157340</t>
+          <t>9204000968</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -8935,28 +9626,28 @@
       </c>
       <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="4" t="n">
-        <v>1032995.69</v>
+        <v>3657989.45</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>крупные штрафы/неустойки 1 032 996 ₽</t>
+          <t>крупные штрафы/неустойки 3 657 989 ₽</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>ОООПолимерспецстрой</t>
+          <t>Ресурс-Дон</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>6155050037</t>
+          <t>6163138292</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -8971,28 +9662,28 @@
       </c>
       <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="4" t="n">
-        <v>0</v>
+        <v>18336806.38</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>крупные штрафы/неустойки 18 336 806 ₽</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>ОООПКТ</t>
+          <t>АМЕТИСТ</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>6168032645</t>
+          <t>6165157340</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -9007,11 +9698,11 @@
       </c>
       <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="4" t="n">
-        <v>0</v>
+        <v>1032995.69</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>крупные штрафы/неустойки 1 032 996 ₽</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete all 67 companies (final 15: group 6 tail + group 7)
All NOSTROY + arbitration checks done. Final 15 (ДОНЮГСТРОЙ, Доммастер,
Горизонт, Альянс-Т, Ника, Айрапетян Игнат, Кошаташян, Ремстрой, Санрайз-Строй,
АСМ-Инжиниринг, Гнатюк, Южпромгеология, Цыбанев, Строй Альянс Юг, Налбандян)
all действителен, no подряд cases 2025+.

Report: 67/67 checked, 0 pending. Risk: 44 high, 3 medium, 20 low.
16 приостановлено, 13 ОДО не установлен, 32 with подряд cases 2025+.

https://claude.ai/code/session_01Uw6wTDP1sFGwQhdVkqv1x9
</commit_message>
<xml_diff>
--- a/audit/audit_report_corrected.xlsx
+++ b/audit/audit_report_corrected.xlsx
@@ -507,7 +507,7 @@
     <row r="1" ht="95" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 52/67; дела проверены: 52/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 16, ОДО не установлен: 12. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 43, Средний: 1, Низкий: 8, Ожидает: 15.</t>
+          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 67/67; дела проверены: 67/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 16, ОДО не установлен: 13. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 44, Средний: 3, Низкий: 20, Ожидает: 0.</t>
         </is>
       </c>
     </row>
@@ -3670,36 +3670,38 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I55" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K55" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L55" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L55" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -3727,36 +3729,38 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I56" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K56" s="4" t="n">
         <v>765551.85</v>
       </c>
-      <c r="L56" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>Средний</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены; небольшие штрафы/неустойки 765 552 ₽</t>
+          <t>небольшие штрафы/неустойки 765 552 ₽</t>
         </is>
       </c>
     </row>
@@ -3784,36 +3788,38 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I57" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K57" s="4" t="n">
         <v>5000</v>
       </c>
-      <c r="L57" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L57" s="7" t="inlineStr">
+        <is>
+          <t>Средний</t>
         </is>
       </c>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены; небольшие штрафы/неустойки 5 000 ₽</t>
+          <t>небольшие штрафы/неустойки 5 000 ₽</t>
         </is>
       </c>
     </row>
@@ -3841,36 +3847,38 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I58" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K58" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L58" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L58" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -3898,36 +3906,38 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K59" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L59" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -3955,36 +3965,38 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I60" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K60" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L60" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L60" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4012,36 +4024,38 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K61" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L61" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L61" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M61" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4069,36 +4083,38 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I62" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K62" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L62" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L62" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4126,36 +4142,38 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I63" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K63" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L63" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L63" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M63" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4183,36 +4201,38 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I64" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K64" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L64" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L64" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4240,36 +4260,38 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I65" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K65" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L65" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L65" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M65" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4297,36 +4319,38 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I66" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K66" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L66" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L66" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4354,36 +4378,38 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I67" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K67" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L67" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L67" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M67" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -4411,36 +4437,38 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>не установлен</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K68" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L68" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>уровень ответственности (ОДО) не установлен</t>
         </is>
       </c>
     </row>
@@ -4468,36 +4496,38 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="inlineStr"/>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>⏳ не проверено (kad)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K69" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L69" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="L69" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M69" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -13626,154 +13656,154 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Строй Альянс Юг</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>6168058072</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>не установлен</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>уровень ответственности (ОДО) не установлен</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>Средний</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>СК Сварог</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>6165150168</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>действителен</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>Второй уровень</t>
         </is>
       </c>
-      <c r="F45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="4" t="n">
+      <c r="F46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="4" t="n">
         <v>303572.19</v>
       </c>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t>небольшие штрафы/неустойки 303 572 ₽</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>Гаджиева Лала Гамид Кызы</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>614909563219</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>ДОММАСТЕР</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0800019547</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>действителен</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Первый уровень</t>
         </is>
       </c>
-      <c r="F46" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>ИНКОМ</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>0816030754</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="F47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>765551.85</v>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>небольшие штрафы/неустойки 765 552 ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>СК ГОРИЗОНТ</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>6141047940</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>действителен</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>Второй уровень</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>АРИАЛ</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>6166065317</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>действителен</t>
-        </is>
-      </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F48" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+          <t>небольшие штрафы/неустойки 5 000 ₽</t>
         </is>
       </c>
     </row>
@@ -13785,12 +13815,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>ДВР</t>
+          <t>Гаджиева Лала Гамид Кызы</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>6163207475</t>
+          <t>614909563219</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -13800,7 +13830,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Третий уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
@@ -13823,12 +13853,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>ЭЛЕМЕНТ СИТИ СТРОЙ</t>
+          <t>ИНКОМ</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>6143099278</t>
+          <t>0816030754</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -13861,12 +13891,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Патриот</t>
+          <t>АРИАЛ</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>0816027053</t>
+          <t>6166065317</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -13876,7 +13906,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
@@ -13899,12 +13929,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>НОЙОН</t>
+          <t>ДВР</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>0816037238</t>
+          <t>6163207475</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -13914,7 +13944,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Третий уровень</t>
         </is>
       </c>
       <c r="F52" s="3" t="n">
@@ -13937,544 +13967,572 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
+          <t>ЭЛЕМЕНТ СИТИ СТРОЙ</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>6143099278</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Патриот</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0816027053</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>НОЙОН</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0816037238</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
           <t>ТАМАРА</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>6166129874</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>действителен</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>Первый уровень</t>
         </is>
       </c>
-      <c r="F53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="F56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>СК ДОНЮГСТРОЙ</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>6163211048</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr"/>
-      <c r="G54" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>ДОММАСТЕР</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>0800019547</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr"/>
-      <c r="G55" s="4" t="n">
-        <v>765551.85</v>
-      </c>
-      <c r="H55" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены; небольшие штрафы/неустойки 765 552 ₽</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>СК ГОРИЗОНТ</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>6141047940</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr"/>
-      <c r="G56" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены; небольшие штрафы/неустойки 5 000 ₽</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Альянс-Т</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>6162074590</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr"/>
-      <c r="G57" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>НИКА</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>0816034124</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr"/>
-      <c r="G58" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Айрапетян Игнат Аршавирович</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>615522305969</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr"/>
-      <c r="G59" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>Кошаташян Амлет Грандович</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>610200085371</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr"/>
-      <c r="G60" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>РемСтрой</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>0816010067</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr"/>
-      <c r="G61" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>САНРАЙЗ-СТРОЙ</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
         <is>
           <t>0800015937</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F62" s="3" t="inlineStr"/>
-      <c r="G62" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>АСМ-Инжиниринг</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>6165187104</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr"/>
-      <c r="G63" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>Гнатюк Юрий Степанович</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>612802867122</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F64" s="3" t="inlineStr"/>
-      <c r="G64" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>ОООЮЖПРОМГЕОЛОГИЯ</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>6155064061</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr"/>
-      <c r="G65" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>Цыбанев Игорь Николаевич</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>080500824511</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr"/>
-      <c r="G66" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>Строй Альянс Юг</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>6168058072</t>
-        </is>
-      </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr"/>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G67" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>⏳ ожидает данных</t>
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -14489,21 +14547,23 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>⏳ ожидает данных</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr"/>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="G68" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>ожидается проверка: НОСТРОЙ не проверен, дела по подряду не проверены</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-verify 4 thin records: full case cards, all anomalies cleared
Айрапетян Игорь & СтройГарант: подряд cases confirmed real & 2025+ →
verdicts stay Высокий on solid evidence. АМЕТИСТ: full UUID + 2nd case found.
Триумф: full card. Audit now clean: 0 placeholder URLs, 0 broken UUIDs,
0 bad dates. 92 подряд cases total. Risk unchanged: 44 high, 3 medium, 20 low.

https://claude.ai/code/session_01Uw6wTDP1sFGwQhdVkqv1x9
</commit_message>
<xml_diff>
--- a/audit/audit_report_corrected.xlsx
+++ b/audit/audit_report_corrected.xlsx
@@ -2327,11 +2327,11 @@
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>А53-36865/2025 — 1 459 508 ₽ — истец</t>
+          <t>А53-36865/2025 — 1 459 508 ₽ — истец; А53-5236/2025 — 197 833 ₽ — истец</t>
         </is>
       </c>
       <c r="K32" s="4" t="n">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1); крупные штрафы/неустойки 1 032 996 ₽</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (2); крупные штрафы/неустойки 1 032 996 ₽</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>А53-42304/2025 — 0 ₽ — истец</t>
+          <t>А53-42304/2025 — 172 276 ₽ — ответчик</t>
         </is>
       </c>
       <c r="K34" s="4" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>А53-17299/2025 — 0 ₽ — истец</t>
+          <t>А53-17299/2025 — 300 000 ₽ — ответчик</t>
         </is>
       </c>
       <c r="K35" s="4" t="n">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>А59-4019/2025 — 0 ₽ — истец</t>
+          <t>А59-4019/2025 — 102 949 ₽ — истец</t>
         </is>
       </c>
       <c r="K36" s="4" t="n">
@@ -6255,7 +6255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11463,44 +11463,44 @@
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/517f59bb-51d1-49c5-955c-3ba6165b</t>
+          <t>https://kad.arbitr.ru/Card/517f59bb-51d1-49c5-955c-3ba6165b6f89</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Триумф</t>
+          <t>АМЕТИСТ</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>6154097900</t>
+          <t>6165157340</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>А53-42304/2025</t>
+          <t>А53-5236/2025</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>20.02.2025</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>ООО "Триумф"</t>
+          <t>ООО "Аметист"</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ФГБОУ ВО "Российская Академия Народного Хозяйства и Государственной Службы При Президенте Российской Федерации" (РАНХиГС)</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr"/>
@@ -11510,11 +11510,11 @@
         </is>
       </c>
       <c r="J85" s="4" t="n">
-        <v>0</v>
+        <v>197833.32</v>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Выиграно</t>
         </is>
       </c>
       <c r="L85" s="3" t="inlineStr">
@@ -11524,29 +11524,29 @@
       </c>
       <c r="M85" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card?number=А53-42304/2025</t>
+          <t>https://kad.arbitr.ru/Card/c0cf2f60-4d12-4d10-b56b-ed198ab3c5f3</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>АЙРАПЕТЯН ИГОРЬ АРШАВИРОВИЧ</t>
+          <t>Триумф</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>615509586157</t>
+          <t>6154097900</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>А53-17299/2025</t>
+          <t>А53-42304/2025</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>21.05.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
@@ -11556,26 +11556,26 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>ИП Айрапетян И. А.</t>
+          <t>НКО "Фонд Капитального Ремонта"</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ООО "Триумф"</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>истец</t>
+          <t>ответчик</t>
         </is>
       </c>
       <c r="J86" s="4" t="n">
-        <v>0</v>
+        <v>172275.5</v>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Частично проиграно</t>
         </is>
       </c>
       <c r="L86" s="3" t="inlineStr">
@@ -11585,29 +11585,29 @@
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card?number=А53-17299/2025</t>
+          <t>https://kad.arbitr.ru/Card/f29291b7-396e-4217-9810-f39f11850a61</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>СтройГарант</t>
+          <t>АЙРАПЕТЯН ИГОРЬ АРШАВИРОВИЧ</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>6153028043</t>
+          <t>615509586157</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>А59-4019/2025</t>
+          <t>А53-17299/2025</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21.05.2025</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
@@ -11617,26 +11617,30 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>ООО "СтройГарант"</t>
+          <t>НКО "Фонд Капитального Ремонта"</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H87" s="3" t="inlineStr"/>
+          <t>ИП Айрапетян И. А.</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Стройлидер"</t>
+        </is>
+      </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>истец</t>
+          <t>ответчик</t>
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Не проиграно</t>
         </is>
       </c>
       <c r="L87" s="3" t="inlineStr">
@@ -11646,44 +11650,44 @@
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card?number=А59-4019/2025</t>
+          <t>https://kad.arbitr.ru/Card/311ec147-5568-4e01-9ea9-fc928bfd0dd9</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>Сериков Владимир Николаевич</t>
+          <t>СтройГарант</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>615430629307</t>
+          <t>6153028043</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>А53-16785/2026</t>
+          <t>А59-4019/2025</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>04.05.2026</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>ИП Сериков В. Н.</t>
+          <t>ООО "Стройгарант"</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>ИП Убейкина И. А.</t>
+          <t>ООО "СК "Монолит"</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr"/>
@@ -11693,21 +11697,21 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>230000</v>
+        <v>102948.71</v>
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Выиграно</t>
         </is>
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>Рассматривается</t>
+          <t>Завершено</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/d332ec56-460d-4699-8e4d-52981633f0dd</t>
+          <t>https://kad.arbitr.ru/Card/85d334dc-1476-4925-b739-ff2f9076bee9</t>
         </is>
       </c>
     </row>
@@ -11724,17 +11728,17 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>А53-156/2025</t>
+          <t>А53-16785/2026</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>09.01.2025</t>
+          <t>04.05.2026</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -11744,7 +11748,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>ИП Магомаева Б. К.</t>
+          <t>ИП Убейкина И. А.</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr"/>
@@ -11754,104 +11758,104 @@
         </is>
       </c>
       <c r="J89" s="4" t="n">
-        <v>2150000</v>
+        <v>230000</v>
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>Выиграно</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L89" s="3" t="inlineStr">
         <is>
-          <t>Завершено</t>
+          <t>Рассматривается</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/ed23e9ea-66a1-4ecc-9e79-2437dd220672</t>
+          <t>https://kad.arbitr.ru/Card/d332ec56-460d-4699-8e4d-52981633f0dd</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Войтиков Виталий Геннадьевич</t>
+          <t>Сериков Владимир Николаевич</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>613302494379</t>
+          <t>615430629307</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>А53-11209/2026</t>
+          <t>А53-156/2025</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>26.03.2026</t>
+          <t>09.01.2025</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам строительного подряда</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>ИП Кочнев С. Ф.</t>
+          <t>ИП Сериков В. Н.</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>ИП Войтиков В. Г.</t>
+          <t>ИП Магомаева Б. К.</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr"/>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>ответчик</t>
+          <t>истец</t>
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>1085929</v>
+        <v>2150000</v>
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Выиграно</t>
         </is>
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>Рассматривается</t>
+          <t>Завершено</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/82a38280-30c4-4bcd-ac79-f6ed2acd62ae</t>
+          <t>https://kad.arbitr.ru/Card/ed23e9ea-66a1-4ecc-9e79-2437dd220672</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>ВЕРТИКАЛЬ 61</t>
+          <t>Войтиков Виталий Геннадьевич</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>6101932201</t>
+          <t>613302494379</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>А53-17329/2025</t>
+          <t>А53-11209/2026</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>21.05.2025</t>
+          <t>26.03.2026</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
@@ -11861,12 +11865,12 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>АО "Тагмет"</t>
+          <t>ИП Кочнев С. Ф.</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>ООО "Вертикаль-61"</t>
+          <t>ИП Войтиков В. Г.</t>
         </is>
       </c>
       <c r="H91" s="3" t="inlineStr"/>
@@ -11876,43 +11880,43 @@
         </is>
       </c>
       <c r="J91" s="4" t="n">
-        <v>2907192.54</v>
+        <v>1085929</v>
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>Частично проиграно</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L91" s="3" t="inlineStr">
         <is>
-          <t>Завершено</t>
+          <t>Рассматривается</t>
         </is>
       </c>
       <c r="M91" s="3" t="inlineStr">
         <is>
-          <t>https://kad.arbitr.ru/Card/cade9cad-35ac-4394-9488-e208232c05b6</t>
+          <t>https://kad.arbitr.ru/Card/82a38280-30c4-4bcd-ac79-f6ed2acd62ae</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>Галеян Араик Дереникович</t>
+          <t>ВЕРТИКАЛЬ 61</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>182900235059</t>
+          <t>6101932201</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>А53-20020/2026</t>
+          <t>А53-17329/2025</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>25.05.2026</t>
+          <t>21.05.2025</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
@@ -11922,34 +11926,95 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>ИП Галеян А. Д.</t>
+          <t>АО "Тагмет"</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>ООО "Ортус"</t>
+          <t>ООО "Вертикаль-61"</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr"/>
       <c r="I92" s="3" t="inlineStr">
         <is>
+          <t>ответчик</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="n">
+        <v>2907192.54</v>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>Частично проиграно</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t>Завершено</t>
+        </is>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>https://kad.arbitr.ru/Card/cade9cad-35ac-4394-9488-e208232c05b6</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Галеян Араик Дереникович</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>182900235059</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>А53-20020/2026</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>25.05.2026</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>О неисполнении или ненадлежащем исполнении обязательств по договорам подряда</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>ИП Галеян А. Д.</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>ООО "Ортус"</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr"/>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
           <t>истец</t>
         </is>
       </c>
-      <c r="J92" s="4" t="n">
+      <c r="J93" s="4" t="n">
         <v>7268993.26</v>
       </c>
-      <c r="K92" s="3" t="inlineStr">
+      <c r="K93" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L92" s="3" t="inlineStr">
+      <c r="L93" s="3" t="inlineStr">
         <is>
           <t>Рассматривается</t>
         </is>
       </c>
-      <c r="M92" s="3" t="inlineStr">
+      <c r="M93" s="3" t="inlineStr">
         <is>
           <t>https://kad.arbitr.ru/Card/7105a8f7-9d7b-4722-863b-2ce14df7f088</t>
         </is>
@@ -12713,12 +12778,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Сериков Владимир Николаевич</t>
+          <t>АМЕТИСТ</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>615430629307</t>
+          <t>6165157340</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -12735,11 +12800,11 @@
         <v>2</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0</v>
+        <v>1032995.69</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (2)</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (2); крупные штрафы/неустойки 1 032 996 ₽</t>
         </is>
       </c>
     </row>
@@ -12751,12 +12816,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>МЕРКУРИЙ</t>
+          <t>Сериков Владимир Николаевич</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>6168115080</t>
+          <t>615430629307</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -12766,18 +12831,18 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (2)</t>
         </is>
       </c>
     </row>
@@ -12789,17 +12854,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>КОМПАНИЯ ДДК</t>
+          <t>МЕРКУРИЙ</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>6168081843</t>
+          <t>6168115080</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Приостановлено</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -12827,22 +12892,22 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Барабанов Алексей Михайлович</t>
+          <t>КОМПАНИЯ ДДК</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>343527639881</t>
+          <t>6168081843</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>Приостановлено</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="F23" s="3" t="n">
@@ -12853,7 +12918,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>арбитражные дела по подряду 2025+ (1)</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>
@@ -12865,12 +12930,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>ЮгСтрой</t>
+          <t>Барабанов Алексей Михайлович</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>6168103663</t>
+          <t>343527639881</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -12903,33 +12968,33 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>СТРОЙГАРАНТ</t>
+          <t>ЮгСтрой</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>9204000968</t>
+          <t>6168103663</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>приостановлен</t>
+          <t>действителен</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Третий уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>3657989.45</v>
+        <v>0</v>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1); крупные штрафы/неустойки 3 657 989 ₽</t>
+          <t>арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>
@@ -12941,12 +13006,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Сизенко Максим Алексеевич</t>
+          <t>СТРОЙГАРАНТ</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>615520155429</t>
+          <t>9204000968</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -12956,18 +13021,18 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Третий уровень</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>527700.48</v>
+        <v>3657989.45</v>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1); крупные штрафы/неустойки 3 657 989 ₽</t>
         </is>
       </c>
     </row>
@@ -12979,12 +13044,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>АМЕТИСТ</t>
+          <t>Сизенко Максим Алексеевич</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>6165157340</t>
+          <t>615520155429</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -13001,11 +13066,11 @@
         <v>1</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>1032995.69</v>
+        <v>527700.48</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1); крупные штрафы/неустойки 1 032 996 ₽</t>
+          <t>статус НОСТРОЙ приостановлен; арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix 7 NOSTROY errors flagged by client (status + ОДО), both audits
Client ground-truth corrections (extension misread reestr.nostroy.ru):
- ОДО "не установлен" → "Первый уровень": Строй Альянс Юг, ВЕРТИКАЛЬ 61, Мегаполис
- статус "действителен" → "приостановлен": НОЙОН, Айрапетян Игнат,
  АСМ-Инжиниринг, Южпромгеология

Applied to both audit/ and audit_2026-05-21/ (same INNs reused). Risk recalc:
ОДО fix moved Мегаполис & Строй Альянс Юг High→Low (false ОДО flag removed);
status fix moved the 4 suspended companies →High. Each record annotated
with correction_note.

https://claude.ai/code/session_01Uw6wTDP1sFGwQhdVkqv1x9
</commit_message>
<xml_diff>
--- a/audit/audit_report_corrected.xlsx
+++ b/audit/audit_report_corrected.xlsx
@@ -507,7 +507,7 @@
     <row r="1" ht="95" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 67/67; дела проверены: 67/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 16, ОДО не установлен: 13. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 44, Средний: 3, Низкий: 20, Ожидает: 0.</t>
+          <t>Проверка членов СРО (исправленная методика). Компаний: 67. НОСТРОЙ проверено: 67/67; дела проверены: 67/67. Фильтр контрактов: дата окончания ≥ 01.01.2023 (цифры из выверенной выгрузки ЦИСК). НОСТРОЙ (reestr.nostroy.ru): статус права + уровень КФ ОДО (обеспечение договорных обязательств, не путать с КФ ВВ); приостановлено: 20, ОДО не установлен: 10. Суды: берутся ТОЛЬКО дела категории «…по договорам подряда», затем дата ≥ 01.01.2025. Описание = № дела + сумма иска + роль (истец/ответчик/третье лицо). Риск — Высокий: 46, Средний: 3, Низкий: 18, Ожидает: 0.</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -3104,14 +3104,14 @@
       <c r="K45" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L45" s="5" t="inlineStr">
-        <is>
-          <t>Высокий</t>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t>уровень ответственности (ОДО) не установлен</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -3163,14 +3163,14 @@
       <c r="K46" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L46" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t>уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (1)</t>
+          <t>арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -3989,14 +3989,14 @@
       <c r="K60" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L60" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
+      <c r="L60" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -4225,14 +4225,14 @@
       <c r="K64" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L64" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -4343,14 +4343,14 @@
       <c r="K66" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L66" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4442,7 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
@@ -4461,14 +4461,14 @@
       <c r="K68" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="L68" s="5" t="inlineStr">
-        <is>
-          <t>Высокий</t>
+      <c r="L68" s="6" t="inlineStr">
+        <is>
+          <t>Низкий</t>
         </is>
       </c>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t>уровень ответственности (ОДО) не установлен</t>
+          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -13249,7 +13249,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F32" s="3" t="n">
@@ -13260,7 +13260,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>уровень ответственности (ОДО) не установлен; арбитражные дела по подряду 2025+ (1)</t>
+          <t>арбитражные дела по подряду 2025+ (1)</t>
         </is>
       </c>
     </row>
@@ -13576,22 +13576,22 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Мегаполис</t>
+          <t>НОЙОН</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>6164280527</t>
+          <t>0816037238</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F41" s="3" t="n">
@@ -13602,7 +13602,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>уровень ответственности (ОДО) не установлен</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
@@ -13728,22 +13728,22 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Строй Альянс Юг</t>
+          <t>Айрапетян Игнат Аршавирович</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>6168058072</t>
+          <t>615522305969</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>не установлен</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
@@ -13754,29 +13754,29 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>уровень ответственности (ОДО) не установлен</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>Средний</t>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>СК Сварог</t>
+          <t>АСМ-Инжиниринг</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>6165150168</t>
+          <t>6165187104</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -13788,33 +13788,33 @@
         <v>0</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>303572.19</v>
+        <v>0</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>небольшие штрафы/неустойки 303 572 ₽</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>Средний</t>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Высокий</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>ДОММАСТЕР</t>
+          <t>ОООЮЖПРОМГЕОЛОГИЯ</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>0800019547</t>
+          <t>6155064061</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>действителен</t>
+          <t>приостановлен</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -13826,11 +13826,11 @@
         <v>0</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>765551.85</v>
+        <v>0</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>небольшие штрафы/неустойки 765 552 ₽</t>
+          <t>статус НОСТРОЙ приостановлен</t>
         </is>
       </c>
     </row>
@@ -13842,109 +13842,109 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
+          <t>СК Сварог</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>6165150168</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Второй уровень</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>303572.19</v>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>небольшие штрафы/неустойки 303 572 ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>ДОММАСТЕР</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0800019547</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>действителен</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Первый уровень</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>765551.85</v>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>небольшие штрафы/неустойки 765 552 ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
           <t>СК ГОРИЗОНТ</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>6141047940</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>действителен</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>Первый уровень</t>
         </is>
       </c>
-      <c r="F48" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="4" t="n">
+      <c r="F50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="4" t="n">
         <v>5000</v>
       </c>
-      <c r="H48" s="3" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>небольшие штрафы/неустойки 5 000 ₽</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Гаджиева Лала Гамид Кызы</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>614909563219</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>действителен</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Первый уровень</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>Низкий</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>ИНКОМ</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>0816030754</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>действителен</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>Второй уровень</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>НОСТРОЙ действителен; дел по подряду 2025+ нет; штрафов нет</t>
         </is>
       </c>
     </row>
@@ -13956,12 +13956,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>АРИАЛ</t>
+          <t>Гаджиева Лала Гамид Кызы</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>6166065317</t>
+          <t>614909563219</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -13971,7 +13971,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F51" s="3" t="n">
@@ -13994,12 +13994,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>ДВР</t>
+          <t>ИНКОМ</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>6163207475</t>
+          <t>0816030754</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -14009,7 +14009,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Третий уровень</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="F52" s="3" t="n">
@@ -14032,12 +14032,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>ЭЛЕМЕНТ СИТИ СТРОЙ</t>
+          <t>АРИАЛ</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>6143099278</t>
+          <t>6166065317</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -14070,12 +14070,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Патриот</t>
+          <t>ДВР</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>0816027053</t>
+          <t>6163207475</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -14085,7 +14085,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Третий уровень</t>
         </is>
       </c>
       <c r="F54" s="3" t="n">
@@ -14108,12 +14108,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>НОЙОН</t>
+          <t>ЭЛЕМЕНТ СИТИ СТРОЙ</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>0816037238</t>
+          <t>6143099278</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="F55" s="3" t="n">
@@ -14146,12 +14146,12 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>ТАМАРА</t>
+          <t>Патриот</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>6166129874</t>
+          <t>0816027053</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -14184,12 +14184,12 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>СК ДОНЮГСТРОЙ</t>
+          <t>Мегаполис</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>6163211048</t>
+          <t>6164280527</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -14222,12 +14222,12 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Альянс-Т</t>
+          <t>ТАМАРА</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>6162074590</t>
+          <t>6166129874</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F58" s="3" t="n">
@@ -14260,12 +14260,12 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>НИКА</t>
+          <t>СК ДОНЮГСТРОЙ</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>0816034124</t>
+          <t>6163211048</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -14275,7 +14275,7 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F59" s="3" t="n">
@@ -14298,12 +14298,12 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Айрапетян Игнат Аршавирович</t>
+          <t>Альянс-Т</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>615522305969</t>
+          <t>6162074590</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="F60" s="3" t="n">
@@ -14336,12 +14336,12 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Кошаташян Амлет Грандович</t>
+          <t>НИКА</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>610200085371</t>
+          <t>0816034124</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -14374,12 +14374,12 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>РемСтрой</t>
+          <t>Кошаташян Амлет Грандович</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>0816010067</t>
+          <t>610200085371</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Первый уровень</t>
+          <t>Второй уровень</t>
         </is>
       </c>
       <c r="F62" s="3" t="n">
@@ -14412,12 +14412,12 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>САНРАЙЗ-СТРОЙ</t>
+          <t>РемСтрой</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>0800015937</t>
+          <t>0816010067</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -14427,7 +14427,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Второй уровень</t>
+          <t>Первый уровень</t>
         </is>
       </c>
       <c r="F63" s="3" t="n">
@@ -14450,12 +14450,12 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>АСМ-Инжиниринг</t>
+          <t>САНРАЙЗ-СТРОЙ</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>6165187104</t>
+          <t>0800015937</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -14526,12 +14526,12 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>ОООЮЖПРОМГЕОЛОГИЯ</t>
+          <t>Цыбанев Игорь Николаевич</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>6155064061</t>
+          <t>080500824511</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -14564,12 +14564,12 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Цыбанев Игорь Николаевич</t>
+          <t>Строй Альянс Юг</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>080500824511</t>
+          <t>6168058072</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">

</xml_diff>